<commit_message>
style: Diseno ejecutivo profesional con colores corporativos y bordes en Excel
</commit_message>
<xml_diff>
--- a/docs/Matriz_Responsabilidades.xlsx
+++ b/docs/Matriz_Responsabilidades.xlsx
@@ -1,58 +1,275 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Matriz Responsabilidades" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Matriz de Responsabilidades" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+  <si>
+    <t>COLEGIO UNIVERSITARIO DE CARTAGO</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN V — TAREA CORTA 2: ARQUITECTURA DE API GATEWAYS Y MICROSERVICIOS</t>
+  </si>
+  <si>
+    <t>Docente: Prof. Ing. Gabriel González Solano   |   Fecha: 15 de Octubre de 2026   |   Periodo: III Cuatrimestre 2026</t>
+  </si>
+  <si>
+    <t>Miembro del Equipo</t>
+  </si>
+  <si>
+    <t>Rol en el Proyecto</t>
+  </si>
+  <si>
+    <t>Módulo / Responsabilidad</t>
+  </si>
+  <si>
+    <t>% Participación</t>
+  </si>
+  <si>
+    <t>Entregables Concretos</t>
+  </si>
+  <si>
+    <t>Héctor Román Arrieta</t>
+  </si>
+  <si>
+    <t>Backend Developer</t>
+  </si>
+  <si>
+    <t>Microservicio de Productos / Catálogo</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Desarrollo de API REST en puerto 5001, modelo NoSQL en MongoDB (cuc_productos_db), endpoints CRUD, control de inventario y endpoint de descuento de stock.</t>
+  </si>
+  <si>
+    <t>Ramsés Aguilar Monge</t>
+  </si>
+  <si>
+    <t>Líder Técnico &amp; Arquitectura</t>
+  </si>
+  <si>
+    <t>API Gateway Centralizado y Enrutamiento</t>
+  </si>
+  <si>
+    <t>Diseño del Gateway en puerto 8080, middleware de enrutamiento perimetral, política de transformación de cabeceras (X-Gateway, X-Request-Id), observabilidad y logging estructurado.</t>
+  </si>
+  <si>
+    <t>Alejandro Morales</t>
+  </si>
+  <si>
+    <t>Backend &amp; Documentación</t>
+  </si>
+  <si>
+    <t>Microservicio de Clientes e Investigación</t>
+  </si>
+  <si>
+    <t>Desarrollo de API REST en puerto 5002, modelo NoSQL en MongoDB (cuc_clientes_db), scripts de seed de datos y redacción formal del informe teórico en formato APA 7ma edición.</t>
+  </si>
+  <si>
+    <t>Fabián Espinoza Méndez</t>
+  </si>
+  <si>
+    <t>Microservicio de Órdenes e Inter-Servicio</t>
+  </si>
+  <si>
+    <t>Desarrollo de API REST en puerto 5003, modelo NoSQL en MongoDB (cuc_ordenes_db), comunicación inter-servicio con Productos y Clientes para validación de stock y precios.</t>
+  </si>
+  <si>
+    <t>José Rodolfo Morales Calderón</t>
+  </si>
+  <si>
+    <t>Backend &amp; Integración BFF</t>
+  </si>
+  <si>
+    <t>Política de Agregación y Pruebas Postman</t>
+  </si>
+  <si>
+    <t>Implementación del endpoint de agregación BFF (/api/resumen-orden/:id), agregación de dashboard (/api/dashboard) y diseño de la colección completa de pruebas en Postman v2.1.</t>
+  </si>
+  <si>
+    <t>TOTAL DE PARTICIPACIÓN DEL EQUIPO:</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Todos los requerimientos funcionales, gateway y teóricos cubiertos de forma equitativa.</t>
+  </si>
+  <si>
+    <t>📌 Arquitectura: 3 Microservicios independientes (5001, 5002, 5003) + API Gateway centralizado (8080) con Entrada Única.</t>
+  </si>
+  <si>
+    <t>🍃 Base de Datos: Persistencia NoSQL aislada en MongoDB (cuc_productos_db, cuc_clientes_db, cuc_ordenes_db).</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
-    <font>
-      <sz val="12"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="15" x14ac:knownFonts="1">
+    <font>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF334155"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF334155"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF166534"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF003366"/>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF065F46"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B2545"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF134074"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2E8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCBD5E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0FDF4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -60,18 +277,125 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF002244"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF002244"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF94A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF94A3B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF003366"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF003366"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="19">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,121 +720,188 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:E15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="48.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="80.83203125" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Miembro del Equipo</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Rol en el Proyecto</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Módulo / Tarea Asignada</v>
-      </c>
-      <c r="D1" t="str">
-        <v>% Participación</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Entregables Concretos</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Héctor Román Arrieta</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Microservicio de Productos / Catálogo</v>
-      </c>
-      <c r="D2" t="str">
-        <v>20%</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Desarrollo de API REST en puerto 5001, modelo NoSQL en MongoDB (cuc_productos_db), endpoints CRUD, lógica de validación de stock y endpoint de descuento de inventario.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Ramsés Aguilar Monge</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Líder Técnico &amp; Arquitectura</v>
-      </c>
-      <c r="C3" t="str">
-        <v>API Gateway Centralizado y Enrutamiento</v>
-      </c>
-      <c r="D3" t="str">
-        <v>20%</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Diseño del Gateway en puerto 8080, middleware de enrutamiento perimetral, política de transformación de cabeceras (X-Gateway, X-Request-Id), observabilidad y logging de tráfico.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Alejandro Morales</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Backend &amp; Documentación</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Microservicio de Clientes e Investigación Teórica</v>
-      </c>
-      <c r="D4" t="str">
-        <v>20%</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Desarrollo de API REST en puerto 5002, modelo NoSQL en MongoDB (cuc_clientes_db), scripts de seed de datos y redacción formal del documento de investigación teórica en formato APA.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Fabián Espinoza Méndez</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Microservicio de Órdenes y Comunicación Inter-Servicio</v>
-      </c>
-      <c r="D5" t="str">
-        <v>20%</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Desarrollo de API REST en puerto 5003, modelo NoSQL en MongoDB (cuc_ordenes_db), comunicación inter-servicio con Productos y Clientes para validación de stock y precios.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>José Rodolfo Morales Calderón</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Backend &amp; Integración</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Política de Agregación y Pruebas Postman</v>
-      </c>
-      <c r="D6" t="str">
-        <v>20%</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Endpoint de agregación BFF (/api/resumen-orden/:id), agregación de dashboard general (/api/dashboard) y diseño de la colección completa de pruebas en Postman v2.1.</v>
-      </c>
+    <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
-  </ignoredErrors>
+  <mergeCells count="6">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Agregar documento formal PDF de investigacion y actualizar dependencias
</commit_message>
<xml_diff>
--- a/docs/Matriz_Responsabilidades.xlsx
+++ b/docs/Matriz_Responsabilidades.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0EFF68-BE25-49B9-A1FD-7446B561D4BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Matriz de Responsabilidades" state="visible" r:id="rId4"/>
+    <sheet name="Matriz de Responsabilidades" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -115,94 +124,94 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.5"/>
+      <color rgb="FF334155"/>
+      <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
+      <sz val="10.5"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+      <color rgb="FF0F172A"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF334155"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FF166534"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF475569"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FF0F172A"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FF003366"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <i/>
-      <color rgb="FF334155"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
+      <color rgb="FF64748B"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10.5"/>
+      <sz val="9"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="FF334155"/>
-      <sz val="9.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF166534"/>
-      <sz val="10.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="FF475569"/>
       <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="10.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF003366"/>
-      <sz val="11"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF64748B"/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1E3A8A"/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF065F46"/>
-      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
@@ -328,6 +337,42 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -337,44 +382,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
@@ -720,9 +729,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:E15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -731,150 +740,150 @@
     <col min="5" max="5" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+    </row>
+    <row r="3" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" spans="1:5" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+    <row r="12" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="15" t="s">
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>31</v>
       </c>
@@ -883,7 +892,7 @@
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
     </row>
-    <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>32</v>
       </c>
@@ -894,14 +903,14 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: corregir inventario, configuracion y pruebas del gateway
- Ordenes: validar stock antes de descontar, compensar reservas fallidas
  y devolver stock al cancelar (solo PENDIENTE/PAGADA)
- Productos: descuento atomico y endpoint reponer-stock
- Validacion de IDs (400) en todos los servicios
- Corregir /health capturado por /:id y lectura de .env por servicio
- Configuracion centralizada en config.js y .env.example
- Pruebas automatizadas con node:test (npm test)
- Limpieza: script Excel movido a tools/, dependencias de docs en devDependencies
- Documento de investigacion sin nombres del equipo y con link al repo, en PDF
</commit_message>
<xml_diff>
--- a/docs/Matriz_Responsabilidades.xlsx
+++ b/docs/Matriz_Responsabilidades.xlsx
@@ -1,26 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0EFF68-BE25-49B9-A1FD-7446B561D4BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Matriz de Responsabilidades" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Matriz de Responsabilidades" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>COLEGIO UNIVERSITARIO DE CARTAGO</t>
   </si>
@@ -46,7 +37,7 @@
     <t>Entregables Concretos</t>
   </si>
   <si>
-    <t>Héctor Román Arrieta</t>
+    <t>[Nombre omitido]</t>
   </si>
   <si>
     <t>Backend Developer</t>
@@ -73,9 +64,6 @@
     <t>Diseño del Gateway en puerto 8080, middleware de enrutamiento perimetral, política de transformación de cabeceras (X-Gateway, X-Request-Id), observabilidad y logging estructurado.</t>
   </si>
   <si>
-    <t>Alejandro Morales</t>
-  </si>
-  <si>
     <t>Backend &amp; Documentación</t>
   </si>
   <si>
@@ -83,9 +71,6 @@
   </si>
   <si>
     <t>Desarrollo de API REST en puerto 5002, modelo NoSQL en MongoDB (cuc_clientes_db), scripts de seed de datos y redacción formal del informe teórico en formato APA 7ma edición.</t>
-  </si>
-  <si>
-    <t>Fabián Espinoza Méndez</t>
   </si>
   <si>
     <t>Microservicio de Órdenes e Inter-Servicio</t>
@@ -124,94 +109,94 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="15" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF334155"/>
+      <sz val="9.5"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF334155"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF166534"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="10.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF003366"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <i/>
-      <sz val="9.5"/>
-      <color rgb="FF334155"/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <sz val="10.5"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF0F172A"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="9.5"/>
-      <color rgb="FF334155"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="9.5"/>
-      <color rgb="FF1E293B"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.5"/>
-      <color rgb="FF166534"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
+      <color rgb="FF065F46"/>
       <sz val="9"/>
-      <color rgb="FF475569"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.5"/>
-      <color rgb="FF0F172A"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF003366"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF64748B"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF1E3A8A"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF065F46"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
@@ -337,6 +322,15 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -367,23 +361,14 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
@@ -729,9 +714,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -740,161 +725,161 @@
     <col min="5" max="5" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+    <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-    </row>
-    <row r="3" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-    </row>
-    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-    </row>
-    <row r="5" spans="1:5" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="5" t="s">
+    </row>
+    <row r="10" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="E10" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="9" t="s">
+    </row>
+    <row r="11" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="B11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="E11" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="4" t="s">
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="E12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="11" t="s">
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
         <v>29</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>31</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
     </row>
-    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="18"/>
@@ -903,14 +888,14 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>